<commit_message>
modified: al2o3 structured and random lammps file
</commit_message>
<xml_diff>
--- a/structural_analysis/calc.xlsx
+++ b/structural_analysis/calc.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
   <si>
     <t xml:space="preserve">Slag System</t>
   </si>
@@ -261,6 +261,27 @@
   </si>
   <si>
     <t xml:space="preserve">ionic r</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ionic r(A)</t>
+  </si>
+  <si>
+    <t>D(cm2/s)</t>
+  </si>
+  <si>
+    <t>visc</t>
+  </si>
+  <si>
+    <t>visc(poise)</t>
+  </si>
+  <si>
+    <t>diff</t>
+  </si>
+  <si>
+    <t>Mg&lt;Al&lt;Ca&lt;Si&lt;O</t>
+  </si>
+  <si>
+    <t>O&lt;Ca&lt;Al&lt;Si&lt;Mg</t>
   </si>
 </sst>
 </file>
@@ -283,7 +304,6 @@
     </font>
     <font>
       <sz val="12.000000"/>
-      <color indexed="64"/>
       <name val="Times New Roman"/>
     </font>
   </fonts>
@@ -447,7 +467,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -497,11 +517,14 @@
     <xf fontId="0" fillId="0" borderId="10" numFmtId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf fontId="1" fillId="3" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5695,11 +5718,11 @@
         <v>8.9253000000000002e-10</v>
       </c>
       <c r="E43">
-        <f>($B$40*B43)/(6*3.14*$D$40*D43)</f>
+        <f t="shared" ref="E43:E52" si="17">($B$40*B43)/(6*3.14*$D$40*D43)</f>
         <v>0.012448089601278498</v>
       </c>
       <c r="F43" s="22">
-        <f t="shared" ref="F43:F52" si="17">E43*10</f>
+        <f t="shared" ref="F43:F52" si="18">E43*10</f>
         <v>0.12448089601278498</v>
       </c>
     </row>
@@ -5719,11 +5742,11 @@
         <v>9.2023999999999992e-10</v>
       </c>
       <c r="E44">
-        <f t="shared" ref="E44:E52" si="18">($B$40*B44)/(6*3.14*$D$40*D44)</f>
+        <f t="shared" si="17"/>
         <v>0.012145421647137802</v>
       </c>
       <c r="F44" s="22">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0.12145421647137802</v>
       </c>
     </row>
@@ -5743,11 +5766,11 @@
         <v>9.0935999999999995e-10</v>
       </c>
       <c r="E45">
+        <f t="shared" si="17"/>
+        <v>0.012363763769348857</v>
+      </c>
+      <c r="F45" s="22">
         <f t="shared" si="18"/>
-        <v>0.012363763769348857</v>
-      </c>
-      <c r="F45" s="22">
-        <f t="shared" si="17"/>
         <v>0.12363763769348857</v>
       </c>
     </row>
@@ -5767,11 +5790,11 @@
         <v>1.0234e-09</v>
       </c>
       <c r="E46">
+        <f t="shared" si="17"/>
+        <v>0.011115820823491357</v>
+      </c>
+      <c r="F46" s="22">
         <f t="shared" si="18"/>
-        <v>0.011115820823491357</v>
-      </c>
-      <c r="F46" s="22">
-        <f t="shared" si="17"/>
         <v>0.11115820823491357</v>
       </c>
     </row>
@@ -5791,11 +5814,11 @@
         <v>1.0624e-09</v>
       </c>
       <c r="E47">
+        <f t="shared" si="17"/>
+        <v>0.010832784111659484</v>
+      </c>
+      <c r="F47" s="22">
         <f t="shared" si="18"/>
-        <v>0.010832784111659484</v>
-      </c>
-      <c r="F47" s="22">
-        <f t="shared" si="17"/>
         <v>0.10832784111659484</v>
       </c>
     </row>
@@ -5815,11 +5838,11 @@
         <v>1.1429999999999999e-09</v>
       </c>
       <c r="E48">
+        <f t="shared" si="17"/>
+        <v>0.010185099431052504</v>
+      </c>
+      <c r="F48" s="22">
         <f t="shared" si="18"/>
-        <v>0.010185099431052504</v>
-      </c>
-      <c r="F48" s="22">
-        <f t="shared" si="17"/>
         <v>0.10185099431052504</v>
       </c>
     </row>
@@ -5839,11 +5862,11 @@
         <v>1.2092999999999997e-09</v>
       </c>
       <c r="E49">
+        <f t="shared" si="17"/>
+        <v>0.0097365314307111504</v>
+      </c>
+      <c r="F49" s="22">
         <f t="shared" si="18"/>
-        <v>0.0097365314307111504</v>
-      </c>
-      <c r="F49" s="22">
-        <f t="shared" si="17"/>
         <v>0.097365314307111511</v>
       </c>
     </row>
@@ -5863,11 +5886,11 @@
         <v>1.2991999999999998e-09</v>
       </c>
       <c r="E50">
+        <f t="shared" si="17"/>
+        <v>0.0091650294555303043</v>
+      </c>
+      <c r="F50" s="22">
         <f t="shared" si="18"/>
-        <v>0.0091650294555303043</v>
-      </c>
-      <c r="F50" s="22">
-        <f t="shared" si="17"/>
         <v>0.091650294555303047</v>
       </c>
     </row>
@@ -5887,11 +5910,11 @@
         <v>1.2925e-09</v>
       </c>
       <c r="E51">
+        <f t="shared" si="17"/>
+        <v>0.0093152998669949316</v>
+      </c>
+      <c r="F51" s="22">
         <f t="shared" si="18"/>
-        <v>0.0093152998669949316</v>
-      </c>
-      <c r="F51" s="22">
-        <f t="shared" si="17"/>
         <v>0.093152998669949319</v>
       </c>
     </row>
@@ -5911,11 +5934,11 @@
         <v>1.4146999999999999e-09</v>
       </c>
       <c r="E52">
+        <f t="shared" si="17"/>
+        <v>0.0086045408125800006</v>
+      </c>
+      <c r="F52" s="22">
         <f t="shared" si="18"/>
-        <v>0.0086045408125800006</v>
-      </c>
-      <c r="F52" s="22">
-        <f t="shared" si="17"/>
         <v>0.086045408125799999</v>
       </c>
     </row>
@@ -5938,7 +5961,7 @@
         <v>0.40000000000000002</v>
       </c>
       <c r="D58" t="e">
-        <f>1/(B58*C58)</f>
+        <f t="shared" ref="D58:D62" si="19">1/(B58*C58)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -5949,8 +5972,8 @@
       <c r="B59" s="26">
         <v>0.53500000000000003</v>
       </c>
-      <c r="D59" s="27" t="e">
-        <f>1/(B59*C59)</f>
+      <c r="D59" s="17" t="e">
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -5961,8 +5984,8 @@
       <c r="B60" s="26">
         <v>1</v>
       </c>
-      <c r="D60" s="27" t="e">
-        <f>1/(B60*C60)</f>
+      <c r="D60" s="17" t="e">
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -5973,8 +5996,8 @@
       <c r="B61" s="26">
         <v>0.71999999999999997</v>
       </c>
-      <c r="D61" s="27" t="e">
-        <f>1/(B61*C61)</f>
+      <c r="D61" s="17" t="e">
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
       <c r="G61" t="s">
@@ -5988,8 +6011,8 @@
       <c r="B62" s="26">
         <v>1.3999999999999999</v>
       </c>
-      <c r="D62" s="27" t="e">
-        <f>1/(B62*C62)</f>
+      <c r="D62" s="17" t="e">
+        <f t="shared" si="19"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -6010,6 +6033,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
+    <col bestFit="1" min="7" max="8" width="11.421875"/>
     <col bestFit="1" min="11" max="11" width="17.8515625"/>
     <col bestFit="1" min="12" max="12" width="10.3515625"/>
     <col bestFit="1" min="13" max="13" width="12.640625"/>
@@ -6019,7 +6043,7 @@
       <c r="L5" t="s">
         <v>52</v>
       </c>
-      <c r="M5" s="28">
+      <c r="M5" s="27">
         <f>1.380649*10^(-23)</f>
         <v>1.3806490000000001e-23</v>
       </c>
@@ -6089,19 +6113,19 @@
       <c r="I8" s="15">
         <v>6002</v>
       </c>
-      <c r="J8" s="29">
-        <f>(D8*$D$12+E8*$E$12+F8*$F$12+G8*$G$12+H8*$H$12)/(D8+E8+F8+G8+H8)</f>
+      <c r="J8" s="28">
+        <f t="shared" ref="J8:J9" si="20">(D8*$D$12+E8*$E$12+F8*$F$12+G8*$G$12+H8*$H$12)/(D8+E8+F8+G8+H8)</f>
         <v>1.1112262579140284</v>
       </c>
       <c r="K8" s="9">
         <v>1.3801000000000001e-05</v>
       </c>
       <c r="L8">
-        <f>K8*10^(-4)</f>
+        <f t="shared" ref="L8:L9" si="21">K8*10^(-4)</f>
         <v>1.3801e-09</v>
       </c>
       <c r="M8">
-        <f>($M$5*$M$6)/(6*3.14*J8*10^(-10)*L8)</f>
+        <f t="shared" ref="M8:M9" si="22">($M$5*$M$6)/(6*3.14*J8*10^(-10)*L8)</f>
         <v>0.0087111602268108036</v>
       </c>
       <c r="N8">
@@ -6131,19 +6155,19 @@
       <c r="I9" s="15">
         <v>6000</v>
       </c>
-      <c r="J9" s="29">
-        <f>(D9*$D$12+E9*$E$12+F9*$F$12+G9*$G$12+H9*$H$12)/(D9+E9+F9+G9+H9)</f>
+      <c r="J9" s="28">
+        <f t="shared" si="20"/>
         <v>1.1086266666666666</v>
       </c>
       <c r="K9" s="9">
         <v>1.3876000000000001e-05</v>
       </c>
       <c r="L9">
-        <f>K9*10^(-4)</f>
+        <f t="shared" si="21"/>
         <v>1.3875999999999998e-09</v>
       </c>
       <c r="M9">
-        <f>($M$5*$M$6)/(6*3.14*J9*10^(-10)*L9)</f>
+        <f t="shared" si="22"/>
         <v>0.0086843924457949521</v>
       </c>
       <c r="N9">
@@ -6173,23 +6197,23 @@
       <c r="I10" s="15">
         <v>6000</v>
       </c>
-      <c r="J10" s="29">
-        <f>(D10*$D$12+E10*$E$12+F10*$F$12+G10*$G$12+H10*$H$12)/(D10+E10+F10+G10+H10)</f>
+      <c r="J10" s="28">
+        <f t="shared" ref="J10:J11" si="23">(D10*$D$12+E10*$E$12+F10*$F$12+G10*$G$12+H10*$H$12)/(D10+E10+F10+G10+H10)</f>
         <v>1.1060566666666667</v>
       </c>
       <c r="K10" s="9">
         <v>1.4812e-05</v>
       </c>
       <c r="L10">
-        <f>K10*10^(-4)</f>
+        <f t="shared" ref="L10:L11" si="24">K10*10^(-4)</f>
         <v>1.4811999999999998e-09</v>
       </c>
       <c r="M10">
-        <f>($M$5*$M$6)/(6*3.14*J10*10^(-10)*L10)</f>
+        <f t="shared" ref="M10:M11" si="25">($M$5*$M$6)/(6*3.14*J10*10^(-10)*L10)</f>
         <v>0.0081545119167098327</v>
       </c>
       <c r="N10">
-        <f>M10*10</f>
+        <f t="shared" ref="N10:N11" si="26">M10*10</f>
         <v>0.081545119167098334</v>
       </c>
     </row>
@@ -6215,23 +6239,23 @@
       <c r="I11" s="15">
         <v>5998</v>
       </c>
-      <c r="J11" s="29">
-        <f>(D11*$D$12+E11*$E$12+F11*$F$12+G11*$G$12+H11*$H$12)/(D11+E11+F11+G11+H11)</f>
+      <c r="J11" s="28">
+        <f t="shared" si="23"/>
         <v>1.1035011670556851</v>
       </c>
       <c r="K11" s="9">
         <v>1.5644000000000001e-05</v>
       </c>
       <c r="L11">
-        <f>K11*10^(-4)</f>
+        <f t="shared" si="24"/>
         <v>1.5644000000000001e-09</v>
       </c>
       <c r="M11">
-        <f>($M$5*$M$6)/(6*3.14*J11*10^(-10)*L11)</f>
+        <f t="shared" si="25"/>
         <v>0.0077387078003221289</v>
       </c>
       <c r="N11">
-        <f>M11*10</f>
+        <f t="shared" si="26"/>
         <v>0.077387078003221282</v>
       </c>
     </row>
@@ -6255,29 +6279,132 @@
         <v>0.53500000000000003</v>
       </c>
     </row>
-    <row r="23" ht="14.25">
-      <c r="D23" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="24" ht="14.25">
-      <c r="D24" t="s">
-        <v>63</v>
+    <row r="17" ht="14.25">
+      <c r="D17" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="F17" t="s">
+        <v>82</v>
+      </c>
+      <c r="G17" t="s">
+        <v>83</v>
+      </c>
+      <c r="H17" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="D18" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18" s="19">
+        <v>9.6419230000000002e-05</v>
+      </c>
+      <c r="G18">
+        <f>($M$5*$M$6)/(6*3.14*E18*10^(-10)*F18)</f>
+        <v>1.3855601813745457e-07</v>
+      </c>
+      <c r="H18">
+        <f>G18*10</f>
+        <v>1.3855601813745457e-06</v>
+      </c>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="D19" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E19">
+        <v>0.40000000000000002</v>
+      </c>
+      <c r="F19" s="19">
+        <v>2.215175e-05</v>
+      </c>
+      <c r="G19" s="30">
+        <f>($M$5*$M$6)/(6*3.14*E19*10^(-10)*F19)</f>
+        <v>1.5077211259470928e-06</v>
+      </c>
+      <c r="H19" s="30">
+        <f>G19*10</f>
+        <v>1.5077211259470927e-05</v>
+      </c>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="D20" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="E20">
+        <v>0.71999999999999997</v>
+      </c>
+      <c r="F20" s="19">
+        <v>2.291762e-06</v>
+      </c>
+      <c r="G20" s="30">
+        <f>($M$5*$M$6)/(6*3.14*E20*10^(-10)*F20)</f>
+        <v>8.0963083939825719e-06</v>
+      </c>
+      <c r="H20" s="30">
+        <f>G20*10</f>
+        <v>8.0963083939825716e-05</v>
+      </c>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="D21" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E21">
+        <v>1.3999999999999999</v>
+      </c>
+      <c r="F21" s="19">
+        <v>0.0007592791</v>
+      </c>
+      <c r="G21" s="30">
+        <f>($M$5*$M$6)/(6*3.14*E21*10^(-10)*F21)</f>
+        <v>1.2567808992089064e-08</v>
+      </c>
+      <c r="H21" s="30">
+        <f>G21*10</f>
+        <v>1.2567808992089065e-07</v>
+      </c>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="D22" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E22">
+        <v>0.53500000000000003</v>
+      </c>
+      <c r="F22" s="19">
+        <v>1.7539189999999999e-05</v>
+      </c>
+      <c r="G22" s="30">
+        <f>($M$5*$M$6)/(6*3.14*E22*10^(-10)*F22)</f>
+        <v>1.4237237770413356e-06</v>
+      </c>
+      <c r="H22" s="30">
+        <f>G22*10</f>
+        <v>1.4237237770413357e-05</v>
       </c>
     </row>
     <row r="25" ht="14.25">
       <c r="D25" t="s">
-        <v>64</v>
+        <v>85</v>
+      </c>
+      <c r="E25" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="26" ht="14.25">
       <c r="D26" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="27" ht="14.25">
-      <c r="D27" t="s">
-        <v>67</v>
+        <v>83</v>
+      </c>
+      <c r="E26" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>